<commit_message>
Update Zenodo DOI for submission release
</commit_message>
<xml_diff>
--- a/manuscript_submission_snapshot/additional_files/additional_file_5_survey_design_and_sex_comparator_audits.xlsx
+++ b/manuscript_submission_snapshot/additional_files/additional_file_5_survey_design_and_sex_comparator_audits.xlsx
@@ -1838,6 +1838,7 @@
       <c r="B2" t="n">
         <v>0</v>
       </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>188</v>
       </c>
@@ -1847,6 +1848,7 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>32</v>
       </c>
@@ -1856,6 +1858,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -1883,6 +1886,7 @@
       <c r="B3" t="n">
         <v>0</v>
       </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>178</v>
       </c>
@@ -1892,6 +1896,7 @@
       <c r="F3" t="n">
         <v>0</v>
       </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>0</v>
       </c>
@@ -1901,6 +1906,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>13</v>
       </c>
@@ -1942,6 +1948,7 @@
       <c r="F4" t="n">
         <v>0</v>
       </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>3</v>
       </c>
@@ -1951,6 +1958,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>32</v>
       </c>
@@ -1978,6 +1986,7 @@
       <c r="B5" t="n">
         <v>0</v>
       </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>40</v>
       </c>
@@ -1987,6 +1996,7 @@
       <c r="F5" t="n">
         <v>0</v>
       </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>1</v>
       </c>
@@ -1996,6 +2006,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>4</v>
       </c>
@@ -2023,6 +2034,7 @@
       <c r="B6" t="n">
         <v>0</v>
       </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>99</v>
       </c>
@@ -2032,6 +2044,7 @@
       <c r="F6" t="n">
         <v>0</v>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>7</v>
       </c>
@@ -2041,6 +2054,7 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>19</v>
       </c>
@@ -2068,6 +2082,7 @@
       <c r="B7" t="n">
         <v>0</v>
       </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>95</v>
       </c>
@@ -2077,6 +2092,7 @@
       <c r="F7" t="n">
         <v>0</v>
       </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>0</v>
       </c>
@@ -2086,6 +2102,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>0</v>
       </c>
@@ -2113,6 +2130,7 @@
       <c r="B8" t="n">
         <v>0</v>
       </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>217</v>
       </c>
@@ -2122,6 +2140,7 @@
       <c r="F8" t="n">
         <v>0</v>
       </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>59</v>
       </c>
@@ -2131,6 +2150,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>36</v>
       </c>
@@ -2604,10 +2624,10 @@
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="51" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
@@ -2775,16 +2795,16 @@
         <v>-4.103497573360236</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0165148125026219</v>
+        <v>0.01651481250262199</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0112571369720698</v>
+        <v>0.01125713697206985</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0242280992648001</v>
+        <v>0.02422809926480011</v>
       </c>
       <c r="T2" t="n">
-        <v>8.946384834629071e-98</v>
+        <v>8.946384834629069e-98</v>
       </c>
     </row>
     <row r="3">
@@ -2855,7 +2875,7 @@
         <v>1.253883165646517</v>
       </c>
       <c r="S3" t="n">
-        <v>1.546165427571847</v>
+        <v>1.546165427571848</v>
       </c>
       <c r="T3" t="n">
         <v>5.91984415953546e-10</v>
@@ -2929,7 +2949,7 @@
         <v>1.426346394669971</v>
       </c>
       <c r="S4" t="n">
-        <v>1.852141186738628</v>
+        <v>1.852141186738627</v>
       </c>
       <c r="T4" t="n">
         <v>3.127406073629252e-13</v>
@@ -3000,7 +3020,7 @@
         <v>1.679163331132381</v>
       </c>
       <c r="R5" t="n">
-        <v>1.40291056432927</v>
+        <v>1.402910564329271</v>
       </c>
       <c r="S5" t="n">
         <v>2.009814142334608</v>
@@ -3068,7 +3088,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.055404346508027</v>
+        <v>0.05540434650802703</v>
       </c>
       <c r="Q6" t="n">
         <v>1.056967909565404</v>
@@ -3142,7 +3162,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>-0.1922282916839094</v>
+        <v>-0.1922282916839095</v>
       </c>
       <c r="Q7" t="n">
         <v>0.8251184793015933</v>
@@ -3216,7 +3236,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.0235963525233803</v>
+        <v>0.02359635252338034</v>
       </c>
       <c r="Q8" t="n">
         <v>1.023876949121722</v>
@@ -3228,7 +3248,7 @@
         <v>1.041423309098618</v>
       </c>
       <c r="T8" t="n">
-        <v>0.0064936687204108</v>
+        <v>0.006493668720410871</v>
       </c>
     </row>
     <row r="9">
@@ -3290,7 +3310,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.1072034777462315</v>
+        <v>0.1072034777462316</v>
       </c>
       <c r="Q9" t="n">
         <v>1.11316073487421</v>
@@ -3364,7 +3384,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>-0.2844079069103525</v>
+        <v>-0.2844079069103526</v>
       </c>
       <c r="Q10" t="n">
         <v>0.7524596486071095</v>
@@ -3441,13 +3461,13 @@
         <v>-4.232938742998879</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.0145096875898179</v>
+        <v>0.01450968758981796</v>
       </c>
       <c r="R11" t="n">
-        <v>0.009942952292817799</v>
+        <v>0.009942952292817841</v>
       </c>
       <c r="S11" t="n">
-        <v>0.0211738956151073</v>
+        <v>0.02117389561510736</v>
       </c>
       <c r="T11" t="n">
         <v>8.485997960273625e-107</v>
@@ -3524,7 +3544,7 @@
         <v>1.547917225940261</v>
       </c>
       <c r="T12" t="n">
-        <v>8.807760899623684e-10</v>
+        <v>8.807760899623685e-10</v>
       </c>
     </row>
     <row r="13">
@@ -3586,7 +3606,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.4463267528819087</v>
+        <v>0.4463267528819088</v>
       </c>
       <c r="Q13" t="n">
         <v>1.56256195474933</v>
@@ -3595,10 +3615,10 @@
         <v>1.367055405510203</v>
       </c>
       <c r="S13" t="n">
-        <v>1.786028461310834</v>
+        <v>1.786028461310833</v>
       </c>
       <c r="T13" t="n">
-        <v>5.970574408365835e-11</v>
+        <v>5.970574408365836e-11</v>
       </c>
     </row>
     <row r="14">
@@ -3734,7 +3754,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.056849703742831</v>
+        <v>0.05684970374283101</v>
       </c>
       <c r="Q15" t="n">
         <v>1.058496710345938</v>
@@ -3808,7 +3828,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-0.1817507137664214</v>
+        <v>-0.1817507137664215</v>
       </c>
       <c r="Q16" t="n">
         <v>0.8338091716578511</v>
@@ -3882,7 +3902,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.0319333317703947</v>
+        <v>0.03193333177039473</v>
       </c>
       <c r="Q17" t="n">
         <v>1.032448671485543</v>
@@ -3891,10 +3911,10 @@
         <v>1.014882326850032</v>
       </c>
       <c r="S17" t="n">
-        <v>1.050319067591546</v>
+        <v>1.050319067591545</v>
       </c>
       <c r="T17" t="n">
-        <v>0.0002651243532195</v>
+        <v>0.0002651243532195516</v>
       </c>
     </row>
     <row r="18">
@@ -3956,13 +3976,13 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.1078303737216008</v>
+        <v>0.1078303737216009</v>
       </c>
       <c r="Q18" t="n">
         <v>1.113858789639842</v>
       </c>
       <c r="R18" t="n">
-        <v>0.9761698575362848</v>
+        <v>0.9761698575362847</v>
       </c>
       <c r="S18" t="n">
         <v>1.270968770116749</v>
@@ -4107,13 +4127,13 @@
         <v>-4.241403255801109</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.0143873884848335</v>
+        <v>0.01438738848483359</v>
       </c>
       <c r="R20" t="n">
-        <v>0.0098538229789205</v>
+        <v>0.009853822978920549</v>
       </c>
       <c r="S20" t="n">
-        <v>0.0210067653799274</v>
+        <v>0.02100676537992749</v>
       </c>
       <c r="T20" t="n">
         <v>6.443267105041924e-107</v>
@@ -4187,7 +4207,7 @@
         <v>1.252904659583981</v>
       </c>
       <c r="S21" t="n">
-        <v>1.548377509576308</v>
+        <v>1.548377509576307</v>
       </c>
       <c r="T21" t="n">
         <v>8.574263483901137e-10</v>
@@ -4409,7 +4429,7 @@
         <v>1.053229081658769</v>
       </c>
       <c r="S24" t="n">
-        <v>1.064081520644033</v>
+        <v>1.064081520644034</v>
       </c>
       <c r="T24" t="n">
         <v>2.838307339490361e-105</v>
@@ -4483,7 +4503,7 @@
         <v>0.7722233131920145</v>
       </c>
       <c r="S25" t="n">
-        <v>0.9010533112643376</v>
+        <v>0.9010533112643377</v>
       </c>
       <c r="T25" t="n">
         <v>4.084215785427512e-06</v>
@@ -4548,7 +4568,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.0313960971793385</v>
+        <v>0.03139609717933859</v>
       </c>
       <c r="Q26" t="n">
         <v>1.03189415331224</v>
@@ -4557,10 +4577,10 @@
         <v>1.014340128314962</v>
       </c>
       <c r="S26" t="n">
-        <v>1.049751965752214</v>
+        <v>1.049751965752215</v>
       </c>
       <c r="T26" t="n">
-        <v>0.000335242461664</v>
+        <v>0.0003352424616640282</v>
       </c>
     </row>
     <row r="27">
@@ -4622,13 +4642,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.1078422629350608</v>
+        <v>0.1078422629350609</v>
       </c>
       <c r="Q27" t="n">
         <v>1.11387203262348</v>
       </c>
       <c r="R27" t="n">
-        <v>0.97613346064852</v>
+        <v>0.9761334606485199</v>
       </c>
       <c r="S27" t="n">
         <v>1.271046383592326</v>
@@ -4773,13 +4793,13 @@
         <v>-3.891055281117968</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.0204237818304651</v>
+        <v>0.02042378183046517</v>
       </c>
       <c r="R29" t="n">
-        <v>0.0138469532142183</v>
+        <v>0.01384695321421831</v>
       </c>
       <c r="S29" t="n">
-        <v>0.0301243788294252</v>
+        <v>0.03012437882942521</v>
       </c>
       <c r="T29" t="n">
         <v>9.763833031653026e-86</v>
@@ -4844,7 +4864,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.0532197628600005</v>
+        <v>0.05321976286000053</v>
       </c>
       <c r="Q30" t="n">
         <v>1.054661395057919</v>
@@ -4918,10 +4938,10 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>-0.0848695508350564</v>
+        <v>-0.08486955083505648</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.9186321113774424</v>
+        <v>0.9186321113774425</v>
       </c>
       <c r="R31" t="n">
         <v>0.8473018953970454</v>
@@ -4930,7 +4950,7 @@
         <v>0.9959672705067344</v>
       </c>
       <c r="T31" t="n">
-        <v>0.0395950452248882</v>
+        <v>0.03959504522488828</v>
       </c>
     </row>
     <row r="32">
@@ -4992,7 +5012,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.0152801354031518</v>
+        <v>0.01528013540315184</v>
       </c>
       <c r="Q32" t="n">
         <v>1.015397473557967</v>
@@ -5004,7 +5024,7 @@
         <v>1.03298274750793</v>
       </c>
       <c r="T32" t="n">
-        <v>0.0811243742829269</v>
+        <v>0.08112437428292693</v>
       </c>
     </row>
     <row r="33">
@@ -5066,19 +5086,19 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.08784060934888049</v>
+        <v>0.08784060934888052</v>
       </c>
       <c r="Q33" t="n">
         <v>1.091814083200862</v>
       </c>
       <c r="R33" t="n">
-        <v>0.9555930501009148</v>
+        <v>0.9555930501009147</v>
       </c>
       <c r="S33" t="n">
         <v>1.247453601875665</v>
       </c>
       <c r="T33" t="n">
-        <v>0.1963891849557478</v>
+        <v>0.1963891849557479</v>
       </c>
     </row>
     <row r="34">
@@ -5214,7 +5234,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.1348307812226016</v>
+        <v>0.1348307812226017</v>
       </c>
       <c r="Q35" t="n">
         <v>1.144343123621957</v>
@@ -5226,7 +5246,7 @@
         <v>1.207712450188807</v>
       </c>
       <c r="T35" t="n">
-        <v>9.433718787309112e-07</v>
+        <v>9.433718787309111e-07</v>
       </c>
     </row>
     <row r="36">
@@ -5288,7 +5308,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.1432379600901722</v>
+        <v>0.1432379600901723</v>
       </c>
       <c r="Q36" t="n">
         <v>1.154004375981218</v>
@@ -5439,16 +5459,16 @@
         <v>-4.062255248666856</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.017210162120544</v>
+        <v>0.01721016212054405</v>
       </c>
       <c r="R38" t="n">
-        <v>0.0116972557950681</v>
+        <v>0.01169725579506811</v>
       </c>
       <c r="S38" t="n">
-        <v>0.0253212963283483</v>
+        <v>0.02532129632834831</v>
       </c>
       <c r="T38" t="n">
-        <v>1.860009906608852e-94</v>
+        <v>1.860009906608851e-94</v>
       </c>
     </row>
     <row r="39">
@@ -5510,7 +5530,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.055335683136645</v>
+        <v>0.05533568313664506</v>
       </c>
       <c r="Q39" t="n">
         <v>1.056895337076855</v>
@@ -5584,10 +5604,10 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>-0.0804826304119455</v>
+        <v>-0.08048263041194556</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.9226709298585328</v>
+        <v>0.9226709298585327</v>
       </c>
       <c r="R40" t="n">
         <v>0.8500050683134338</v>
@@ -5596,7 +5616,7 @@
         <v>1.001548904284992</v>
       </c>
       <c r="T40" t="n">
-        <v>0.0544820093532651</v>
+        <v>0.05448200935326513</v>
       </c>
     </row>
     <row r="41">
@@ -5658,7 +5678,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.0234549740167059</v>
+        <v>0.02345497401670594</v>
       </c>
       <c r="Q41" t="n">
         <v>1.02373220515972</v>
@@ -5670,7 +5690,7 @@
         <v>1.04164680489662</v>
       </c>
       <c r="T41" t="n">
-        <v>0.008050785645673001</v>
+        <v>0.008050785645673013</v>
       </c>
     </row>
     <row r="42">
@@ -5732,19 +5752,19 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.0862184083891244</v>
+        <v>0.08621840838912444</v>
       </c>
       <c r="Q42" t="n">
         <v>1.090044377144737</v>
       </c>
       <c r="R42" t="n">
-        <v>0.9547855767868112</v>
+        <v>0.9547855767868111</v>
       </c>
       <c r="S42" t="n">
         <v>1.244464488187554</v>
       </c>
       <c r="T42" t="n">
-        <v>0.2021378360415688</v>
+        <v>0.2021378360415689</v>
       </c>
     </row>
     <row r="43">
@@ -5954,7 +5974,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.1517389434915643</v>
+        <v>0.1517389434915644</v>
       </c>
       <c r="Q45" t="n">
         <v>1.16385636449113</v>
@@ -6105,13 +6125,13 @@
         <v>-4.066667423526982</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.0171343951473789</v>
+        <v>0.01713439514737894</v>
       </c>
       <c r="R47" t="n">
-        <v>0.0116401499996287</v>
+        <v>0.0116401499996288</v>
       </c>
       <c r="S47" t="n">
-        <v>0.0252219685378526</v>
+        <v>0.02522196853785262</v>
       </c>
       <c r="T47" t="n">
         <v>1.99232566852508e-94</v>
@@ -6176,7 +6196,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.0554139074327197</v>
+        <v>0.05541390743271971</v>
       </c>
       <c r="Q48" t="n">
         <v>1.056978015204299</v>
@@ -6188,7 +6208,7 @@
         <v>1.062639849465824</v>
       </c>
       <c r="T48" t="n">
-        <v>6.987725590639449e-92</v>
+        <v>6.98772559063945e-92</v>
       </c>
     </row>
     <row r="49">
@@ -6250,10 +6270,10 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>-0.07991635755858489</v>
+        <v>-0.07991635755858495</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.9231935613207356</v>
+        <v>0.9231935613207355</v>
       </c>
       <c r="R49" t="n">
         <v>0.8504831616335164</v>
@@ -6262,7 +6282,7 @@
         <v>1.002120194863215</v>
       </c>
       <c r="T49" t="n">
-        <v>0.0562154214851964</v>
+        <v>0.05621542148519645</v>
       </c>
     </row>
     <row r="50">
@@ -6324,7 +6344,7 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.0229701049255135</v>
+        <v>0.02297010492551357</v>
       </c>
       <c r="Q50" t="n">
         <v>1.023235949375048</v>
@@ -6336,7 +6356,7 @@
         <v>1.04113811306728</v>
       </c>
       <c r="T50" t="n">
-        <v>0.0094400810665071</v>
+        <v>0.009440081066507166</v>
       </c>
     </row>
     <row r="51">
@@ -6398,13 +6418,13 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>0.0862657139138512</v>
+        <v>0.08626571391385128</v>
       </c>
       <c r="Q51" t="n">
         <v>1.09009594348565</v>
       </c>
       <c r="R51" t="n">
-        <v>0.9547847232149144</v>
+        <v>0.9547847232149145</v>
       </c>
       <c r="S51" t="n">
         <v>1.244583346497879</v>
@@ -6472,7 +6492,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>-0.2760478765997899</v>
+        <v>-0.27604787659979</v>
       </c>
       <c r="Q52" t="n">
         <v>0.7587766022478897</v>
@@ -6546,7 +6566,7 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>0.1279727545320955</v>
+        <v>0.1279727545320956</v>
       </c>
       <c r="Q53" t="n">
         <v>1.13652203720054</v>
@@ -6558,7 +6578,7 @@
         <v>1.20084828394763</v>
       </c>
       <c r="T53" t="n">
-        <v>5.218502122923911e-06</v>
+        <v>5.21850212292391e-06</v>
       </c>
     </row>
     <row r="54">
@@ -6620,7 +6640,7 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>0.1508635454471038</v>
+        <v>0.1508635454471039</v>
       </c>
       <c r="Q54" t="n">
         <v>1.162837972719738</v>
@@ -6873,7 +6893,7 @@
         <v>47.52941730459476</v>
       </c>
       <c r="G4" t="n">
-        <v>47.52357258021189</v>
+        <v>47.52357258021188</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>

</xml_diff>